<commit_message>
Clearer room locations, Floor 3 stairs note, LKC/LSC names, human voice on map tap
</commit_message>
<xml_diff>
--- a/data/qa/Dataset Jarvis.xlsx
+++ b/data/qa/Dataset Jarvis.xlsx
@@ -30069,17 +30069,17 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>R Baca berada di Lantai 1, di bagian atas gedung, di sebelah kanan Library.</t>
+          <t>R Baca berada di Lantai 1, di samping Klinik, dekat Library (Kanan).</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Reading Room (R Baca) is on Floor 1, at the top of the building, to the right of the Library.</t>
+          <t>Reading Room (R Baca) is on Floor 1, next to the Clinic, near the Library (Right).</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>阅览室（R Baca）位于1楼，在大楼上方，图书馆的右边。</t>
+          <t>阅览室（R Baca）位于1楼，在诊所旁边，靠近图书馆（右）。</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -30114,17 +30114,17 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Library (Kiri) berada di Lantai 1, di sisi kiri atas gedung, tepat di atas ruang APPLE.</t>
+          <t>Library (Kiri) berada di Lantai 1, di seberang ruang APPLE, di sebelah kiri Klinik.</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Library (Left) is on Floor 1, on the upper left side of the building, just above the APPLE room.</t>
+          <t>Library (Left) is on Floor 1, across from the APPLE room, to the left of the Clinic.</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>图书馆（左）位于1楼，在大楼左上方，APPLE 教室正上方。</t>
+          <t>图书馆（左）位于1楼，在 APPLE 教室对面，诊所的左边。</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -30159,17 +30159,17 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Klinik berada di Lantai 1, di bagian tengah atas, di antara Library dan R Baca.</t>
+          <t>Klinik berada di Lantai 1, di antara Library (Kiri) dan R Baca.</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Clinic (Klinik) is on Floor 1, in the upper middle, between the Library and R Baca.</t>
+          <t>Clinic (Klinik) is on Floor 1, between the Library (Left) and the Reading Room.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>诊所（Klinik）位于1楼，在中间偏上，图书馆和阅览室之间。</t>
+          <t>诊所（Klinik）位于1楼，在图书馆（左）和阅览室之间。</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -30204,17 +30204,17 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Library (Kanan) berada di Lantai 1, di sisi kanan tengah, tepat di bawah R Baca.</t>
+          <t>Library (Kanan) berada di Lantai 1, di sebelah kanan eskalator, di samping R Baca.</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Library (Right) is on Floor 1, on the middle right side, just below R Baca.</t>
+          <t>Library (Right) is on Floor 1, to the right of the escalator, next to the Reading Room.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>图书馆（右）位于1楼，在右侧中间，阅览室正下方。</t>
+          <t>图书馆（右）位于1楼，在扶梯右边，阅览室旁边。</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -30249,17 +30249,17 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>APPLE berada di Lantai 1, di sisi kiri gedung, di bawah Library.</t>
+          <t>APPLE berada di Lantai 1, di seberang Library (Kiri), di sebelah kiri eskalator.</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>APPLE is on Floor 1, on the left side of the building, below the Library.</t>
+          <t>APPLE is on Floor 1, across from the Library (Left), to the left of the escalator.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>APPLE位于1楼，在大楼左侧，图书馆下方。</t>
+          <t>APPLE位于1楼，在图书馆（左）对面，扶梯的左边。</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -30294,17 +30294,17 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Gallery Bersama berada di Lantai 1, di tengah gedung (lokasi kiosk ini).</t>
+          <t>Gallery Bersama berada di Lantai 1, di samping eskalator (lokasi kiosk ini).</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Gallery Bersama is on Floor 1, in the middle of the building (where this kiosk is).</t>
+          <t>Gallery Bersama is on Floor 1, next to the escalator (where this kiosk is).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Gallery Bersama位于1楼，在大楼中间（就是本服务台所在的位置）。</t>
+          <t>Gallery Bersama位于1楼，在扶梯旁边（就是本服务台所在的位置）。</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -30339,17 +30339,17 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Admisi berada di Lantai 1, di sebelah kanan Gallery Bersama, dekat ruang Drop Out.</t>
+          <t>Admisi berada di Lantai 1, di sebelah kanan Gallery Bersama, di samping Drop Out.</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Admissions (Admisi) is on Floor 1, to the right of Gallery Bersama, near Drop Out.</t>
+          <t>Admissions (Admisi) is on Floor 1, to the right of Gallery Bersama, next to Drop Out.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>招生处（Admisi）位于1楼，在 Gallery Bersama 右边，靠近 Drop Out。</t>
+          <t>招生处（Admisi）位于1楼，在 Gallery Bersama 右边，Drop Out 旁边。</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -30384,17 +30384,17 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Drop Out berada di Lantai 1, di sisi kanan gedung, di sebelah kanan Admisi.</t>
+          <t>Drop Out berada di Lantai 1, di ujung kanan gedung, di sebelah kanan Admisi.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Drop Out is on Floor 1, on the right side of the building, to the right of Admisi.</t>
+          <t>Drop Out is on Floor 1, at the far right of the building, to the right of Admissions.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Drop Out 区位于1楼，在大楼右侧，招生处的右边。</t>
+          <t>Drop Out 区位于1楼，在大楼最右侧，招生处的右边。</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -30429,17 +30429,17 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>BCA C0111-12 berada di Lantai 1, di sisi kiri bawah gedung, di bawah ruang APPLE.</t>
+          <t>BCA C0111-12 berada di Lantai 1, di sisi kiri gedung, di ujung kiri Gallery Bersama.</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>BCA C0111-12 is on Floor 1, on the lower left side of the building, below the APPLE room.</t>
+          <t>BCA C0111-12 is on Floor 1, on the left side of the building, at the left end of Gallery Bersama.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>BCA C0111-12位于1楼，在大楼左下方，APPLE 教室下方。</t>
+          <t>BCA C0111-12位于1楼，在大楼左侧，Gallery Bersama 的左端。</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -30474,17 +30474,17 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>SSC berada di Lantai 1, di bagian tengah bawah, di bawah Gallery Bersama.</t>
+          <t>SSC berada di Lantai 1, di seberang Gallery Bersama, di sebelah kiri Marketing.</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>SSC is on Floor 1, in the lower middle, below Gallery Bersama.</t>
+          <t>SSC is on Floor 1, across from Gallery Bersama, to the left of Marketing.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>SSC位于1楼，在中间偏下，Gallery Bersama 下方。</t>
+          <t>SSC位于1楼，在 Gallery Bersama 对面，Marketing 的左边。</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -30519,17 +30519,17 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Marketing berada di Lantai 1, di bagian tengah bawah, tepat di bawah Admisi.</t>
+          <t>Marketing berada di Lantai 1, di samping Admisi, di sebelah kanan SSC.</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Marketing is on Floor 1, in the lower middle, just below Admisi.</t>
+          <t>Marketing is on Floor 1, next to Admissions, to the right of SSC.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Marketing位于1楼，在中间偏下，招生处正下方。</t>
+          <t>Marketing位于1楼，在招生处旁边，SSC 的右边。</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -30564,17 +30564,17 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>SDC berada di Lantai 1, di bagian bawah gedung, di sebelah kiri SADC.</t>
+          <t>SDC berada di Lantai 1, di sebelah kiri SADC, dekat SSC.</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>SDC is on Floor 1, at the bottom of the building, to the left of SADC.</t>
+          <t>SDC is on Floor 1, to the left of SADC, near SSC.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>SDC位于1楼，在大楼下方，SADC 的左边。</t>
+          <t>SDC位于1楼，在 SADC 的左边，靠近 SSC。</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -30609,17 +30609,17 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>SADC C0105 berada di Lantai 1, di bagian bawah gedung, di antara SDC dan UKM.</t>
+          <t>SADC C0105 berada di Lantai 1, di antara SDC dan UKM, dekat SSC.</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>SADC C0105 is on Floor 1, at the bottom of the building, between SDC and UKM.</t>
+          <t>SADC C0105 is on Floor 1, between SDC and UKM, near SSC.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>SADC C0105位于1楼，在大楼下方，SDC 和 UKM 之间。</t>
+          <t>SADC C0105位于1楼，在 SDC 和 UKM 之间，靠近 SSC。</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -30654,17 +30654,17 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>UKM C0104 berada di Lantai 1, di bagian bawah gedung, di sebelah kanan SADC.</t>
+          <t>UKM C0104 berada di Lantai 1, di sebelah kanan SADC, dekat Marketing.</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>UKM C0104 is on Floor 1, at the bottom of the building, to the right of SADC.</t>
+          <t>UKM C0104 is on Floor 1, to the right of SADC, near Marketing.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>UKM C0104位于1楼，在大楼下方，SADC 的右边。</t>
+          <t>UKM C0104位于1楼，在 SADC 的右边，靠近 Marketing。</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -30699,17 +30699,17 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>B0201 berada di Lantai 2.</t>
+          <t>B0201 berada di Lantai 2, di sisi kiri gedung, di seberang Studio Fotografi.</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>B0201 is on Floor 2.</t>
+          <t>B0201 is on Floor 2, on the left side of the building, across from the Photography Studio.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>B0201位于2楼。</t>
+          <t>B0201位于2楼，在大楼左侧，摄影工作室对面。</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -30729,37 +30729,37 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Library Lantai 2</t>
+          <t>Library (LKC)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Library</t>
+          <t>Library (LKC)</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>图书馆</t>
+          <t>图书馆（LKC）</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Library Lantai 2 berada di Lantai 2.</t>
+          <t>Library (LKC) berada di Lantai 2, di seberang eskalator, di sisi kanan gedung.</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Library is on Floor 2.</t>
+          <t>Library (LKC) is on Floor 2, across from the escalator, on the right side of the building.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>图书馆位于2楼。</t>
+          <t>图书馆（LKC）位于2楼，在扶梯对面，大楼右侧。</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Dimana lokasi Library Lantai 2? / Where is Library? / 图书馆在哪里？</t>
+          <t>Dimana lokasi Library (LKC)? / Where is Library (LKC)? / 图书馆（LKC）在哪里？</t>
         </is>
       </c>
     </row>
@@ -30789,17 +30789,17 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Toilet (dekat Library) berada di Lantai 2.</t>
+          <t>Toilet (dekat Library) berada di Lantai 2, di dalam area Library (LKC), di sudut kirinya, dekat Greenscreen.</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Toilet (near the Library) is on Floor 2.</t>
+          <t>Toilet (near the Library) is on Floor 2, inside the Library (LKC) area, in its left corner, near the Green Screen Studio.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>洗手间（靠近图书馆）位于2楼。</t>
+          <t>洗手间（靠近图书馆）位于2楼，在图书馆（LKC）内的左侧角落，靠近绿幕工作室。</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
@@ -30834,17 +30834,17 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Studio Fotografi berada di Lantai 2.</t>
+          <t>Studio Fotografi berada di Lantai 2, di sebelah kiri Greenscreen, di seberang B0201.</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Photography Studio is on Floor 2.</t>
+          <t>Photography Studio is on Floor 2, to the left of the Green Screen Studio, across from B0201.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>摄影工作室位于2楼。</t>
+          <t>摄影工作室位于2楼，在绿幕工作室左边，B0201 对面。</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -30879,17 +30879,17 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Greenscreen berada di Lantai 2.</t>
+          <t>Greenscreen berada di Lantai 2, di sebelah kiri eskalator, di samping Studio Fotografi.</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Green Screen Studio is on Floor 2.</t>
+          <t>Green Screen Studio is on Floor 2, to the left of the escalator, next to the Photography Studio.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>绿幕工作室位于2楼。</t>
+          <t>绿幕工作室位于2楼，在扶梯左边，摄影工作室旁边。</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -30924,17 +30924,17 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Binus TV berada di Lantai 2.</t>
+          <t>Binus TV berada di Lantai 2, di ujung kiri gedung, di sebelah kiri area lift.</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Binus TV is on Floor 2.</t>
+          <t>Binus TV is on Floor 2, at the far left of the building, to the left of the lifts.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Binus TV位于2楼。</t>
+          <t>Binus TV位于2楼，在大楼最左侧，电梯区的左边。</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -30969,17 +30969,17 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Binus Radio berada di Lantai 2.</t>
+          <t>Binus Radio berada di Lantai 2, di seberang area lift, di sebelah kiri Amphitheatre.</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Binus Radio is on Floor 2.</t>
+          <t>Binus Radio is on Floor 2, across from the lifts, to the left of the Amphitheatre.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Binus Radio位于2楼。</t>
+          <t>Binus Radio位于2楼，在电梯区对面，阶梯剧场的左边。</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -31014,17 +31014,17 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Amphitheatre berada di Lantai 2.</t>
+          <t>Amphitheatre berada di Lantai 2, dekat eskalator, di sebelah kanan Binus Radio.</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Amphitheatre is on Floor 2.</t>
+          <t>Amphitheatre is on Floor 2, near the escalator, to the right of Binus Radio.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>阶梯剧场位于2楼。</t>
+          <t>阶梯剧场位于2楼，在扶梯附近，Binus Radio 的右边。</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -31059,17 +31059,17 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>C0207 berada di Lantai 2.</t>
+          <t>C0207 berada di Lantai 2, di seberang eskalator, di sebelah kiri Toilet.</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>C0207 is on Floor 2.</t>
+          <t>C0207 is on Floor 2, across from the escalator, to the left of the toilet.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>C0207位于2楼。</t>
+          <t>C0207位于2楼，在扶梯对面，洗手间的左边。</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -31104,17 +31104,17 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Toilet (dekat C0207) berada di Lantai 2.</t>
+          <t>Toilet (dekat C0207) berada di Lantai 2, dekat eskalator, di antara C0207 dan C0201.</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Toilet (near C0207) is on Floor 2.</t>
+          <t>Toilet (near C0207) is on Floor 2, near the escalator, between C0207 and C0201.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>洗手间（靠近 C0207）位于2楼。</t>
+          <t>洗手间（靠近 C0207）位于2楼，在扶梯附近，C0207 和 C0201 之间。</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -31149,17 +31149,17 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>C0201 berada di Lantai 2.</t>
+          <t>C0201 berada di Lantai 2, di sebelah kanan Toilet, di seberang C0203.</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>C0201 is on Floor 2.</t>
+          <t>C0201 is on Floor 2, to the right of the toilet, across from C0203.</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>C0201位于2楼。</t>
+          <t>C0201位于2楼，在洗手间右边，C0203 对面。</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -31194,17 +31194,17 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>C0212 berada di Lantai 2.</t>
+          <t>C0212 berada di Lantai 2, di ujung kiri gedung, dekat Binus TV.</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>C0212 is on Floor 2.</t>
+          <t>C0212 is on Floor 2, at the far left of the building, near Binus TV.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>C0212位于2楼。</t>
+          <t>C0212位于2楼，在大楼最左侧，Binus TV 附近。</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -31239,17 +31239,17 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>C0209 berada di Lantai 2.</t>
+          <t>C0209 berada di Lantai 2, di samping C0207, di sebelah kiri C0206.</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>C0209 is on Floor 2.</t>
+          <t>C0209 is on Floor 2, next to C0207, to the left of C0206.</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>C0209位于2楼。</t>
+          <t>C0209位于2楼，在 C0207 旁边，C0206 的左边。</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -31284,17 +31284,17 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>C0206 berada di Lantai 2.</t>
+          <t>C0206 berada di Lantai 2, di seberang Toilet, di antara C0209 dan C0203.</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>C0206 is on Floor 2.</t>
+          <t>C0206 is on Floor 2, across from the toilet, between C0209 and C0203.</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>C0206位于2楼。</t>
+          <t>C0206位于2楼，在洗手间对面，C0209 和 C0203 之间。</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -31329,17 +31329,17 @@
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>C0203 berada di Lantai 2.</t>
+          <t>C0203 berada di Lantai 2, di seberang C0201, di sebelah kanan C0206.</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>C0203 is on Floor 2.</t>
+          <t>C0203 is on Floor 2, across from C0201, to the right of C0206.</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>C0203位于2楼。</t>
+          <t>C0203位于2楼，在 C0201 对面，C0206 的右边。</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -31374,17 +31374,17 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>C0210 berada di Lantai 2.</t>
+          <t>C0210 berada di Lantai 2, di seberang C0209, di sebelah kiri C0205.</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>C0210 is on Floor 2.</t>
+          <t>C0210 is on Floor 2, across from C0209, to the left of C0205.</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>C0210位于2楼。</t>
+          <t>C0210位于2楼，在 C0209 对面，C0205 的左边。</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -31419,17 +31419,17 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>C0205 berada di Lantai 2.</t>
+          <t>C0205 berada di Lantai 2, di seberang C0206, di antara C0210 dan C0204.</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>C0205 is on Floor 2.</t>
+          <t>C0205 is on Floor 2, across from C0206, between C0210 and C0204.</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>C0205位于2楼。</t>
+          <t>C0205位于2楼，在 C0206 对面，C0210 和 C0204 之间。</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
@@ -31464,17 +31464,17 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>C0204 berada di Lantai 2.</t>
+          <t>C0204 berada di Lantai 2, di seberang C0203, di sebelah kanan C0205.</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>C0204 is on Floor 2.</t>
+          <t>C0204 is on Floor 2, across from C0203, to the right of C0205.</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>C0204位于2楼。</t>
+          <t>C0204位于2楼，在 C0203 对面，C0205 的右边。</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -31509,17 +31509,17 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Kelas Besar B0301 berada di Lantai 3.</t>
+          <t>Kelas Besar B0301 berada di Lantai 3, di sisi kiri gedung, di sebelah kiri B0302. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Large Classroom B0301 is on Floor 3.</t>
+          <t>Large Classroom B0301 is on Floor 3, on the left side of the building, to the left of B0302. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>大教室 B0301位于3楼。</t>
+          <t>大教室 B0301位于3楼，在大楼左侧，B0302 的左边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -31554,17 +31554,17 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>B0302 berada di Lantai 3.</t>
+          <t>B0302 berada di Lantai 3, di sebelah kanan Kelas Besar B0301, di samping Toilet. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>B0302 is on Floor 3.</t>
+          <t>B0302 is on Floor 3, to the right of Large Classroom B0301, next to the toilet. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>B0302位于3楼。</t>
+          <t>B0302位于3楼，在大教室 B0301 右边，洗手间旁边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -31599,17 +31599,17 @@
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Toilet (dekat B0302) berada di Lantai 3.</t>
+          <t>Toilet (dekat B0302) berada di Lantai 3, di samping B0302, di sebelah kiri Library. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Toilet (near B0302) is on Floor 3.</t>
+          <t>Toilet (near B0302) is on Floor 3, next to B0302, to the left of the Library. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>洗手间（靠近 B0302）位于3楼。</t>
+          <t>洗手间（靠近 B0302）位于3楼，在 B0302 旁边，图书馆的左边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -31644,17 +31644,17 @@
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Library Lantai 3 berada di Lantai 3.</t>
+          <t>Library Lantai 3 berada di Lantai 3, di sisi kanan gedung, di sebelah kanan B0302 dan Toilet. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Library is on Floor 3.</t>
+          <t>Library is on Floor 3, on the right side of the building, to the right of B0302 and the toilet. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>图书馆位于3楼。</t>
+          <t>图书馆位于3楼，在大楼右侧，B0302 和洗手间的右边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -31689,17 +31689,17 @@
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Finance berada di Lantai 3.</t>
+          <t>Finance berada di Lantai 3, di sebelah kanan area lift, di samping Rektorat. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Finance is on Floor 3.</t>
+          <t>Finance is on Floor 3, to the right of the lifts, next to the Rectorate. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>财务处（Finance）位于3楼。</t>
+          <t>财务处（Finance）位于3楼，在电梯区右边，校长办公室旁边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -31734,17 +31734,17 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>Rektorat berada di Lantai 3.</t>
+          <t>Rektorat berada di Lantai 3, di sebelah kanan eskalator, di samping Finance. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Rectorate (Rektorat) is on Floor 3.</t>
+          <t>Rectorate (Rektorat) is on Floor 3, to the right of the escalator, next to Finance. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>校长办公室（Rektorat）位于3楼。</t>
+          <t>校长办公室（Rektorat）位于3楼，在扶梯右边，财务处旁边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -31779,17 +31779,17 @@
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>SADC Lantai 3 berada di Lantai 3.</t>
+          <t>SADC Lantai 3 berada di Lantai 3, di sebelah kiri eskalator, di seberang area lift. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>SADC is on Floor 3.</t>
+          <t>SADC is on Floor 3, to the left of the escalator, across from the lifts. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>SADC位于3楼。</t>
+          <t>SADC位于3楼，在扶梯左边，电梯区对面。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -31824,17 +31824,17 @@
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>C0301 berada di Lantai 3.</t>
+          <t>C0301 berada di Lantai 3, di sisi kanan gedung, di sebelah kanan Toilet. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>C0301 is on Floor 3.</t>
+          <t>C0301 is on Floor 3, on the right side of the building, to the right of the toilet. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>C0301位于3楼。</t>
+          <t>C0301位于3楼，在大楼右侧，洗手间的右边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -31869,17 +31869,17 @@
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>C0307 berada di Lantai 3.</t>
+          <t>C0307 berada di Lantai 3, dekat eskalator, di sebelah kiri Toilet. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>C0307 is on Floor 3.</t>
+          <t>C0307 is on Floor 3, near the escalator, to the left of the toilet. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>C0307位于3楼。</t>
+          <t>C0307位于3楼，在扶梯附近，洗手间的左边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
@@ -31914,17 +31914,17 @@
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>Toilet (dekat C0307) berada di Lantai 3.</t>
+          <t>Toilet (dekat C0307) berada di Lantai 3, di antara C0307 dan C0301. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Toilet (near C0307) is on Floor 3.</t>
+          <t>Toilet (near C0307) is on Floor 3, between C0307 and C0301. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>洗手间（靠近 C0307）位于3楼。</t>
+          <t>洗手间（靠近 C0307）位于3楼，在 C0307 和 C0301 之间。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
@@ -31959,17 +31959,17 @@
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>C0302 berada di Lantai 3.</t>
+          <t>C0302 berada di Lantai 3, di ujung kanan gedung, di samping C0301 dan C0303. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>C0302 is on Floor 3.</t>
+          <t>C0302 is on Floor 3, at the far right of the building, next to C0301 and C0303. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>C0302位于3楼。</t>
+          <t>C0302位于3楼，在大楼最右侧，C0301 和 C0303 旁边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
@@ -32004,17 +32004,17 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>C0312 berada di Lantai 3.</t>
+          <t>C0312 berada di Lantai 3, di ujung kiri gedung, dekat SADC. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>C0312 is on Floor 3.</t>
+          <t>C0312 is on Floor 3, at the far left of the building, near SADC. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>C0312位于3楼。</t>
+          <t>C0312位于3楼，在大楼最左侧，靠近 SADC。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
@@ -32049,17 +32049,17 @@
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>C0309 berada di Lantai 3.</t>
+          <t>C0309 berada di Lantai 3, di seberang C0307, di sebelah kiri C0306. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>C0309 is on Floor 3.</t>
+          <t>C0309 is on Floor 3, across from C0307, to the left of C0306. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>C0309位于3楼。</t>
+          <t>C0309位于3楼，在 C0307 对面，C0306 的左边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -32094,17 +32094,17 @@
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>C0306 berada di Lantai 3.</t>
+          <t>C0306 berada di Lantai 3, di seberang Toilet, di antara C0309 dan C0303. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>C0306 is on Floor 3.</t>
+          <t>C0306 is on Floor 3, across from the toilet, between C0309 and C0303. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>C0306位于3楼。</t>
+          <t>C0306位于3楼，在洗手间对面，C0309 和 C0303 之间。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
@@ -32139,17 +32139,17 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>C0303 berada di Lantai 3.</t>
+          <t>C0303 berada di Lantai 3, di sisi kanan gedung, di samping C0302, di sebelah kanan C0306. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>C0303 is on Floor 3.</t>
+          <t>C0303 is on Floor 3, on the right side of the building, next to C0302, to the right of C0306. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>C0303位于3楼。</t>
+          <t>C0303位于3楼，在大楼右侧，C0302 旁边，C0306 的右边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -32184,17 +32184,17 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>C0311 berada di Lantai 3.</t>
+          <t>C0311 berada di Lantai 3, di ujung kiri gedung, di samping C0312. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>C0311 is on Floor 3.</t>
+          <t>C0311 is on Floor 3, at the far left of the building, next to C0312. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>C0311位于3楼。</t>
+          <t>C0311位于3楼，在大楼最左侧，C0312 旁边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -32229,17 +32229,17 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>C0304 berada di Lantai 3.</t>
+          <t>C0304 berada di Lantai 3, di seberang C0303, di sebelah kanan C0305. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>C0304 is on Floor 3.</t>
+          <t>C0304 is on Floor 3, across from C0303, to the right of C0305. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>C0304位于3楼。</t>
+          <t>C0304位于3楼，在 C0303 对面，C0305 的右边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
@@ -32274,17 +32274,17 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>C0305 berada di Lantai 3.</t>
+          <t>C0305 berada di Lantai 3, di seberang C0306, di antara C0310 dan C0304. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>C0305 is on Floor 3.</t>
+          <t>C0305 is on Floor 3, across from C0306, between C0310 and C0304. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>C0305位于3楼。</t>
+          <t>C0305位于3楼，在 C0306 对面，C0310 和 C0304 之间。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
@@ -32319,17 +32319,17 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>C0310 berada di Lantai 3.</t>
+          <t>C0310 berada di Lantai 3, di seberang C0309, di sebelah kiri C0305. Untuk mahasiswa, Lantai 3 hanya bisa diakses lewat tangga darurat dari Lantai 2 atau Lantai 4.</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>C0310 is on Floor 3.</t>
+          <t>C0310 is on Floor 3, across from C0309, to the left of C0305. Students can only reach Floor 3 by the emergency stairs from Floor 2 or Floor 4.</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>C0310位于3楼。</t>
+          <t>C0310位于3楼，在 C0309 对面，C0305 的左边。学生只能从2楼或4楼走紧急楼梯到3楼。</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr">
@@ -32364,17 +32364,17 @@
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>Auditorium B0401 berada di Lantai 4.</t>
+          <t>Auditorium B0401 berada di Lantai 4, dekat eskalator, di sebelah kiri B0402.</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>Auditorium B0401 is on Floor 4.</t>
+          <t>Auditorium B0401 is on Floor 4, near the escalator, to the left of B0402.</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>礼堂 B0401位于4楼。</t>
+          <t>礼堂 B0401位于4楼，在扶梯附近，B0402 的左边。</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr">
@@ -32409,17 +32409,17 @@
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>B0402 berada di Lantai 4.</t>
+          <t>B0402 berada di Lantai 4, di sebelah kanan Auditorium B0401, di samping Toilet.</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>B0402 is on Floor 4.</t>
+          <t>B0402 is on Floor 4, to the right of Auditorium B0401, next to the toilet.</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>B0402位于4楼。</t>
+          <t>B0402位于4楼，在礼堂 B0401 右边，洗手间旁边。</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -32454,17 +32454,17 @@
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>Toilet (dekat B0402) berada di Lantai 4.</t>
+          <t>Toilet (dekat B0402) berada di Lantai 4, di samping B0402, dekat B0403.</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>Toilet (near B0402) is on Floor 4.</t>
+          <t>Toilet (near B0402) is on Floor 4, next to B0402, near B0403.</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>洗手间（靠近 B0402）位于4楼。</t>
+          <t>洗手间（靠近 B0402）位于4楼，在 B0402 旁边，靠近 B0403。</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
@@ -32499,17 +32499,17 @@
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>B0403 berada di Lantai 4.</t>
+          <t>B0403 berada di Lantai 4, di sebelah kanan Toilet (dekat B0402), di samping B0404.</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>B0403 is on Floor 4.</t>
+          <t>B0403 is on Floor 4, to the right of the toilet near B0402, next to B0404.</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>B0403位于4楼。</t>
+          <t>B0403位于4楼，在 B0402 旁洗手间的右边，B0404 旁边。</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -32544,17 +32544,17 @@
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>B0404 berada di Lantai 4.</t>
+          <t>B0404 berada di Lantai 4, di antara B0403 dan B0405.</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>B0404 is on Floor 4.</t>
+          <t>B0404 is on Floor 4, between B0403 and B0405.</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>B0404位于4楼。</t>
+          <t>B0404位于4楼，在 B0403 和 B0405 之间。</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -32589,17 +32589,17 @@
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>B0405 berada di Lantai 4.</t>
+          <t>B0405 berada di Lantai 4, di sebelah kanan B0404, ruang terakhir di deretan B0403–B0405.</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>B0405 is on Floor 4.</t>
+          <t>B0405 is on Floor 4, to the right of B0404, the last room of the B0403–B0405 row.</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>B0405位于4楼。</t>
+          <t>B0405位于4楼，在 B0404 的右边，B0403–B0405 一排的最后一间。</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -32634,17 +32634,17 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>LSC C0407 berada di Lantai 4.</t>
+          <t>LSC C0407 berada di Lantai 4, di sebelah kanan area lift, di sebelah kiri Toilet (dekat LSC).</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>LSC C0407 is on Floor 4.</t>
+          <t>LSC C0407 is on Floor 4, to the right of the lifts, to the left of the toilet near LSC.</t>
         </is>
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>LSC C0407位于4楼。</t>
+          <t>LSC C0407位于4楼，在电梯区右边，LSC 旁洗手间的左边。</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -32679,17 +32679,17 @@
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>Toilet (dekat LSC) berada di Lantai 4.</t>
+          <t>Toilet (dekat LSC) berada di Lantai 4, di sebelah kanan LSC C0407, di seberang C0406.</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>Toilet (near LSC) is on Floor 4.</t>
+          <t>Toilet (near LSC) is on Floor 4, to the right of LSC C0407, across from C0406.</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>洗手间（靠近 LSC）位于4楼。</t>
+          <t>洗手间（靠近 LSC）位于4楼，在 LSC C0407 右边，C0406 对面。</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -32724,17 +32724,17 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>C0401 berada di Lantai 4.</t>
+          <t>C0401 berada di Lantai 4, di sisi kanan gedung, di samping ruang IT.</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>C0401 is on Floor 4.</t>
+          <t>C0401 is on Floor 4, on the right side of the building, next to the IT room.</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>C0401位于4楼。</t>
+          <t>C0401位于4楼，在大楼右侧，IT 部门旁边。</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -32769,17 +32769,17 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>LSC C0408-09 berada di Lantai 4.</t>
+          <t>LSC C0408-09 berada di Lantai 4, di samping LSC C0407, di sebelah kiri C0406.</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>LSC C0408-09 is on Floor 4.</t>
+          <t>LSC C0408-09 is on Floor 4, next to LSC C0407, to the left of C0406.</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>LSC C0408-09位于4楼。</t>
+          <t>LSC C0408-09位于4楼，在 LSC C0407 旁边，C0406 的左边。</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -32814,17 +32814,17 @@
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>IT berada di Lantai 4.</t>
+          <t>IT berada di Lantai 4, di ujung kanan gedung, di antara C0401 dan C0403.</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>IT is on Floor 4.</t>
+          <t>IT is on Floor 4, at the far right of the building, between C0401 and C0403.</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>IT 部门位于4楼。</t>
+          <t>IT 部门位于4楼，在大楼最右侧，C0401 和 C0403 之间。</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -32859,17 +32859,17 @@
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>C0412 berada di Lantai 4.</t>
+          <t>C0412 berada di Lantai 4, di ujung kiri gedung, di samping C0411.</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>C0412 is on Floor 4.</t>
+          <t>C0412 is on Floor 4, at the far left of the building, next to C0411.</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>C0412位于4楼。</t>
+          <t>C0412位于4楼，在大楼最左侧，C0411 旁边。</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr">
@@ -32904,17 +32904,17 @@
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>C0411 berada di Lantai 4.</t>
+          <t>C0411 berada di Lantai 4, di ujung kiri gedung, di samping C0412.</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>C0411 is on Floor 4.</t>
+          <t>C0411 is on Floor 4, at the far left of the building, next to C0412.</t>
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>C0411位于4楼。</t>
+          <t>C0411位于4楼，在大楼最左侧，C0412 旁边。</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -32949,17 +32949,17 @@
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>C0406 berada di Lantai 4.</t>
+          <t>C0406 berada di Lantai 4, di seberang Toilet (dekat LSC), di sebelah kanan LSC C0408-09.</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>C0406 is on Floor 4.</t>
+          <t>C0406 is on Floor 4, across from the toilet near LSC, to the right of LSC C0408-09.</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>C0406位于4楼。</t>
+          <t>C0406位于4楼，在 LSC 旁洗手间对面，LSC C0408-09 的右边。</t>
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr">
@@ -32994,17 +32994,17 @@
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>C0403 berada di Lantai 4.</t>
+          <t>C0403 berada di Lantai 4, di sisi kanan gedung, di samping ruang IT, di sebelah kanan C0406.</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>C0403 is on Floor 4.</t>
+          <t>C0403 is on Floor 4, on the right side of the building, next to the IT room, to the right of C0406.</t>
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>C0403位于4楼。</t>
+          <t>C0403位于4楼，在大楼右侧，IT 部门旁边，C0406 的右边。</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
@@ -33039,17 +33039,17 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>C0410 berada di Lantai 4.</t>
+          <t>C0410 berada di Lantai 4, di seberang LSC C0408-09.</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>C0410 is on Floor 4.</t>
+          <t>C0410 is on Floor 4, across from LSC C0408-09.</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>C0410位于4楼。</t>
+          <t>C0410位于4楼，在 LSC C0408-09 对面。</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">

</xml_diff>